<commit_message>
problema del la subir al drive solucionado
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -1072,18 +1072,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
puliendo errores en el drive. falta verificar si se suben dupicados borra el anterior
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -903,7 +903,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="27" t="n">
-        <v>45253</v>
+        <v>45254</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -1072,18 +1072,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
trabajando en hacer q los archivos q no se puediron guardar queden pendientes a subir
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -1072,18 +1072,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
haciendo los test y agregue la opcion de si un articulo esta activo o no segun un archivo pfd
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -903,7 +903,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="27" t="n">
-        <v>45254</v>
+        <v>45256</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -1072,18 +1072,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
funcion para tesriar los archivos del drive echa
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Hoja3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="144525" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="21">
     <font>
       <name val="Arial"/>
       <sz val="10"/>
@@ -29,29 +29,12 @@
       <name val="Arial Black"/>
       <family val="2"/>
       <i val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial Black"/>
-      <family val="2"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <family val="1"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color indexed="48"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -189,7 +172,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -235,19 +218,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -271,123 +241,97 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="12" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="13" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="12" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="13" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -895,195 +839,197 @@
   <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
   <cols>
-    <col width="12.5703125" customWidth="1" style="17" min="1" max="1"/>
-    <col width="25.42578125" customWidth="1" style="17" min="2" max="2"/>
-    <col width="28.140625" customWidth="1" style="17" min="3" max="3"/>
-    <col width="20.85546875" customWidth="1" style="17" min="4" max="4"/>
+    <col width="12.5703125" customWidth="1" style="24" min="1" max="1"/>
+    <col width="25.42578125" customWidth="1" style="24" min="2" max="2"/>
+    <col width="28.140625" customWidth="1" style="24" min="3" max="3"/>
+    <col width="20.85546875" customWidth="1" style="24" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="n">
-        <v>45266</v>
-      </c>
-      <c r="E1" s="4" t="n"/>
-    </row>
-    <row r="6" ht="22.5" customHeight="1" s="17">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A1" s="30" t="n">
+        <v>45267</v>
+      </c>
+      <c r="E1" s="3" t="n"/>
+    </row>
+    <row r="6" ht="22.5" customHeight="1" s="24">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>LA PAZ 28  -  HAEDO                           4460-2005</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1" s="17">
-      <c r="A7" s="47" t="inlineStr">
+    <row r="7" ht="22.5" customHeight="1" s="24">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>BUENOS AIRES                   luquearti@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>____________________________________________________________________________________</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="41.25" customHeight="1" s="17">
-      <c r="A9" s="28" t="inlineStr">
+    <row r="9" ht="41.25" customHeight="1" s="24">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>"BANQUETAS”</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="41.25" customHeight="1" s="17">
-      <c r="A10" s="31" t="inlineStr">
+    <row r="10" ht="41.25" customHeight="1" s="24">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>"C/escalera rebatible”</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="41.25" customHeight="1" s="17">
-      <c r="A11" s="32" t="inlineStr">
+    <row r="11" ht="41.25" customHeight="1" s="24">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>"Y TAPIZADA"</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n"/>
-      <c r="C11" s="40" t="n"/>
-      <c r="D11" s="40" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1" s="17">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="41" t="n"/>
-      <c r="C12" s="41" t="n"/>
-      <c r="D12" s="41" t="n"/>
+      <c r="B11" s="26" t="n"/>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="24">
+      <c r="A12" s="29" t="n"/>
+      <c r="B12" s="28" t="n"/>
+      <c r="C12" s="28" t="n"/>
+      <c r="D12" s="28" t="n"/>
     </row>
     <row r="23">
-      <c r="C23" s="19" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1" s="17">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="29" t="n"/>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="11" t="n"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="17">
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="11" t="n"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="17">
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="11" t="n"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="17">
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="10" t="n"/>
-      <c r="D27" s="11" t="n"/>
-    </row>
-    <row r="28" ht="18" customHeight="1" s="17">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="C23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="24">
+      <c r="A24" s="13" t="n"/>
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="24">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="24">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="24">
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="24">
+      <c r="A28" s="35" t="inlineStr">
         <is>
           <t>COD.</t>
         </is>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="35" t="inlineStr">
         <is>
           <t>DESCRIPCION</t>
         </is>
       </c>
-      <c r="C28" s="42" t="n"/>
-      <c r="D28" s="34" t="inlineStr">
+      <c r="C28" s="34" t="n"/>
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>PRECIO</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="19.5" customHeight="1" s="17">
-      <c r="A29" s="24" t="inlineStr">
+    <row r="29" ht="19.5" customHeight="1" s="24">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>BAN-10</t>
         </is>
       </c>
-      <c r="B29" s="43" t="inlineStr">
+      <c r="B29" s="33" t="inlineStr">
         <is>
           <t>BANQUETA C/escalera rebatible</t>
         </is>
       </c>
-      <c r="C29" s="42" t="n"/>
-      <c r="D29" s="44" t="n">
-        <v>8715.088</v>
-      </c>
-    </row>
-    <row r="30" ht="19.5" customHeight="1" s="17">
-      <c r="A30" s="24" t="inlineStr">
+      <c r="C29" s="34" t="n"/>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>********</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="19.5" customHeight="1" s="24">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>BAN-12</t>
         </is>
       </c>
-      <c r="B30" s="43" t="inlineStr">
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>BANQUETA TAPIZADA</t>
         </is>
       </c>
-      <c r="C30" s="42" t="n"/>
-      <c r="D30" s="44" t="n">
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="19" t="n">
         <v>3077.813</v>
       </c>
     </row>
-    <row r="31" ht="19.5" customHeight="1" s="17">
-      <c r="A31" s="14" t="n"/>
-      <c r="B31" s="38" t="inlineStr">
+    <row r="31" ht="19.5" customHeight="1" s="24">
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>Envase x 6 unidades</t>
         </is>
       </c>
-      <c r="C31" s="41" t="n"/>
-      <c r="D31" s="45" t="n"/>
-    </row>
-    <row r="32" ht="18.75" customHeight="1" s="17">
-      <c r="A32" s="39" t="inlineStr">
+      <c r="C31" s="28" t="n"/>
+      <c r="D31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="18.75" customHeight="1" s="24">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>Colores: Rojo- Marfil- Blanco- Verde Manzana-Negro</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1" s="17">
-      <c r="A35" s="29" t="n"/>
-      <c r="B35" s="29" t="n"/>
-      <c r="D35" s="29" t="n"/>
-    </row>
-    <row r="36" ht="16.5" customHeight="1" s="17">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="30" t="n"/>
-      <c r="D36" s="46" t="n"/>
-    </row>
-    <row r="37" ht="16.5" customHeight="1" s="17"/>
-    <row r="38" ht="16.5" customHeight="1" s="17"/>
-    <row r="42" ht="19.5" customHeight="1" s="17">
-      <c r="A42" s="7" t="n"/>
+    <row r="35" ht="18" customHeight="1" s="24">
+      <c r="A35" s="31" t="n"/>
+      <c r="B35" s="31" t="n"/>
+      <c r="D35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="24">
+      <c r="A36" s="11" t="n"/>
+      <c r="B36" s="37" t="n"/>
+      <c r="D36" s="21" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="24"/>
+    <row r="38" ht="16.5" customHeight="1" s="24"/>
+    <row r="42" ht="19.5" customHeight="1" s="24">
+      <c r="A42" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n"/>
+      <c r="A44" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n"/>
+      <c r="A46" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
boton ara obtenre precio echo en la vista step1. encontre un bug con el tole-menu de la vista step2
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -903,14 +903,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="27" t="n">
-        <v>45264.64766263525</v>
+        <v>45272</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="17">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -962,16 +958,6 @@
       <c r="C12" s="41" t="n"/>
       <c r="D12" s="41" t="n"/>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23">
       <c r="C23" s="19" t="n"/>
     </row>
@@ -1045,7 +1031,7 @@
       </c>
       <c r="C30" s="42" t="n"/>
       <c r="D30" s="44" t="n">
-        <v>4778.3</v>
+        <v>11266.96</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1" s="17">
@@ -1065,8 +1051,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35" ht="18" customHeight="1" s="17">
       <c r="A35" s="29" t="n"/>
       <c r="B35" s="29" t="n"/>
@@ -1079,34 +1063,29 @@
     </row>
     <row r="37" ht="16.5" customHeight="1" s="17"/>
     <row r="38" ht="16.5" customHeight="1" s="17"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
     <row r="42" ht="19.5" customHeight="1" s="17">
       <c r="A42" s="7" t="n"/>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="5" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="A12:D12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
arregle el bug visual del menu de los links en l vista step2
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -903,7 +903,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="27" t="n">
-        <v>45272</v>
+        <v>45273</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C30" s="42" t="n"/>
       <c r="D30" s="44" t="n">
-        <v>11266.96</v>
+        <v>19960.12</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1" s="17">

</xml_diff>

<commit_message>
agregue un script para subir a google apps scripts voy hay cambiar la forma en q se suben los archivos
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -903,7 +903,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="27" t="n">
-        <v>45286</v>
+        <v>45287</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -1074,18 +1074,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Trabajando en los scripts de google
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
+++ b/LISTAS/ma/BANQUETA ESCALERA Y TAPIZADA DISMAY.xlsx
@@ -1074,18 +1074,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>